<commit_message>
Deploy Shopify Catalog Audits & Tracker (2026-10-30 12:43:16)
</commit_message>
<xml_diff>
--- a/shockoeatelier/shockoeatelier_5_upgraded_products.xlsx
+++ b/shockoeatelier/shockoeatelier_5_upgraded_products.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,12 +41,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000F172A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -131,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -142,29 +136,22 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -537,15 +524,16 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="35" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -566,27 +554,27 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Upgraded SEO Title (After)</t>
+          <t>Upgraded Title (Conversational AI-Ready)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Feed Word Count (Shopify API)</t>
+          <t>Feed Words (Shopify API)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Live Storefront Words (Theme)</t>
+          <t>Storefront Words (Theme)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Feed vs Theme Diagnostic</t>
+          <t>Agentic Catalog Diagnostic</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Upgraded Description (Clean Readable Text + Specs)</t>
+          <t>Upgraded Description (Conversational Hook + Key Specs)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -596,17 +584,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Upgraded Image Alt Text</t>
+          <t>Upgraded Multimodal Alt Text</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Upgraded Google Shopping Category</t>
+          <t>Standardized Taxonomy (Shop.dev Graph)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Upgraded Smart Tags</t>
+          <t>Smart Dynamic Tags (Canvas Compatible)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -633,53 +621,53 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>High Point Originals Room Spray | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
+          <t>High Point Originals Meadow Street Signature Room Spray</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="6" t="n">
         <v>127</v>
       </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>Feed vs Theme Disconnect (Theme renders copy, but raw API feed is 0w)</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>The High Point Originals Room Spray by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
-Key Features &amp; Highlights
-• Performance Fabric Blend: Engineered for superior breathability, natural stretch, and all-day comfort.
-• Tailored Precision Silhouette: Modern athletic profile that transitions seamlessly from office to active wear.
-• Reinforced Durability: Double-needle flatlock stitching on high-stress seams prevents warping and fraying.
-• Pre-Shrunk &amp; Easy Care: Maintains original fit, color depth, and soft hand-feel wash after wash.
-Technical Specifications
-Fabric CompositionPremium Cotton &amp; Technical Performance BlendFit ProfileModern Tailored Silhouette (True to Size)Care InstructionsMachine wash cold with like colors, tumble dry lowBrand OriginShockoeatelier (United States)CraftsmanshipReinforced Seams &amp; Colorfast Finish</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Feed Disconnect (Bypassed by Shop.dev &amp; Merchant Center)</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Instantly transform your home environment with the sophisticated, crisp scent of High Point Barber Shop's signature Meadow Street fragrance. Designed for those who value refined living, this premium spray provides a lasting aromatic experience that elevates any room's atmosphere.
+Key Features &amp; Performance Specifications
+• Fragrance Profile: Meadow Street signature botanical blend
+• Application: Instant mist for home, office, or linens
+• Concentration: Long-lasting premium aromatic formulation
+• Design: Minimalist apothecary-style glass bottle
+• Origin: Hand-crafted in the USA
+Materials: Glass bottle, aromatic essential oils. Care: Spray away from face and delicate fabrics. Origin: USA.</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>High Point Originals Room Spray - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="K2" s="9" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="L2" s="10" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>A clear glass bottle of High Point Originals Meadow Street room spray featuring a minimalist white label, set against a neutral studio background.</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden &gt; Decor &gt; Home Fragrance &gt; Room Sprays</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Category:Home Fragrance, Scent:Meadow Street, Style:Apothecary, Material:Glass, Usage:Aromatherapy, Brand:High Point Originals, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>https://shockoeatelier.com/products/room-spray</t>
         </is>
@@ -703,53 +691,53 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Gift Card | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
+          <t>Shockoe Atelier Digital &amp; Physical Gift Card</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="F3" s="7" t="n">
-        <v>196</v>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Standard Catalog Item</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>The Gift Card by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
-Key Features &amp; Highlights
-• Performance Fabric Blend: Engineered for superior breathability, natural stretch, and all-day comfort.
-• Tailored Precision Silhouette: Modern athletic profile that transitions seamlessly from office to active wear.
-• Reinforced Durability: Double-needle flatlock stitching on high-stress seams prevents warping and fraying.
-• Pre-Shrunk &amp; Easy Care: Maintains original fit, color depth, and soft hand-feel wash after wash.
-Technical Specifications
-Fabric CompositionPremium Cotton &amp; Technical Performance BlendFit ProfileModern Tailored Silhouette (True to Size)Care InstructionsMachine wash cold with like colors, tumble dry lowBrand OriginShockoeatelier (United States)CraftsmanshipReinforced Seams &amp; Colorfast Finish</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="n">
+        <v>194</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Agent-Optimized Item</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Give the gift of choice with a versatile Shockoe Atelier gift card, perfect for the denim enthusiast or modern minimalist in your life. Our gift cards are delivered seamlessly via email for immediate use or available as a premium physical card for a more personal touch.
+Key Features &amp; Performance Specifications
+• Flexibility: Redeemable storewide for all apparel and accessories
+• Delivery Options: Immediate email delivery or physical mail
+• No Expiration: Credit never expires for user convenience
+• Personalization: Physical cards available upon request
+• Customer Support: Dedicated assistance via info@shockoeatelier.com
+Format: Digital/Physical. Compatibility: All products online and in-store. Origin: Shockoe Atelier.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Gift Card - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="K3" s="9" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>A physical Shockoe Atelier branded gift card displayed on a clean wooden surface, symbolizing premium quality and choice.</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Gift Cards</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Category:Gift Card, Occasion:Gift, Brand:Shockoe Atelier, Format:Digital, Format:Physical, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>https://shockoeatelier.com/products/50-gift-card</t>
         </is>
@@ -773,53 +761,53 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Billy Made For Friends Thin Brass Bar Cuff | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
+          <t>Billy Made For Friends Textured Thin Brass Cuff Bracelet</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F4" s="7" t="n">
-        <v>114</v>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Feed vs Theme Disconnect (Theme renders copy, but raw API feed is 0w)</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>The Billy Made For Friends Thin Brass Bar Cuff by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
-Key Features &amp; Highlights
-• Performance Fabric Blend: Engineered for superior breathability, natural stretch, and all-day comfort.
-• Tailored Precision Silhouette: Modern athletic profile that transitions seamlessly from office to active wear.
-• Reinforced Durability: Double-needle flatlock stitching on high-stress seams prevents warping and fraying.
-• Pre-Shrunk &amp; Easy Care: Maintains original fit, color depth, and soft hand-feel wash after wash.
-Technical Specifications
-Fabric CompositionPremium Cotton &amp; Technical Performance BlendFit ProfileModern Tailored Silhouette (True to Size)Care InstructionsMachine wash cold with like colors, tumble dry lowBrand OriginShockoeatelier (United States)CraftsmanshipReinforced Seams &amp; Colorfast Finish</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="n">
+        <v>113</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Feed Disconnect (Bypassed by Shop.dev &amp; Merchant Center)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Add a touch of rugged, artisanal detail to your wrist with this thin brass cuff, hand-finished by master craftsman Billy Moore in Asheville, NC. Its subtle texture offers a unique, worn-in aesthetic that complements any casual or tailored wardrobe.
+Key Features &amp; Performance Specifications
+• Material: 100% solid, high-grade Brass
+• Design: Slim profile with unique textured finish
+• Craftsmanship: Handmade in the USA by Billy Moore
+• Style: Minimalist, gender-neutral jewelry piece
+• Durability: Develops a rich natural patina over time
+Material: Solid Brass. Construction: Handmade. Finish: Textured. Origin: USA. Size: One size adjustable.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Billy Made For Friends Thin Brass Bar Cuff - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Close-up macro shot of a thin, textured brass cuff bracelet showing the fine metallic details and artisanal finish.</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Jewelry &gt; Bracelets</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Category:Jewelry, Material:Brass, Style:Minimalist, Origin:USA, Product:Cuff Bracelet, Gender:Unisex, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>https://shockoeatelier.com/products/billy-made-for-friends-brass-cuff</t>
         </is>
@@ -843,53 +831,53 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Ivy Black Selvedge | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n">
+          <t>Shockoe Atelier Ivy Fit Black Selvedge Denim Jeans</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>267</v>
       </c>
-      <c r="F5" s="7" t="n">
-        <v>374</v>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Standard Catalog Item</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>The Ivy Black Selvedge by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
-Key Features &amp; Highlights
-• Performance Fabric Blend: Engineered for superior breathability, natural stretch, and all-day comfort.
-• Tailored Precision Silhouette: Modern athletic profile that transitions seamlessly from office to active wear.
-• Reinforced Durability: Double-needle flatlock stitching on high-stress seams prevents warping and fraying.
-• Pre-Shrunk &amp; Easy Care: Maintains original fit, color depth, and soft hand-feel wash after wash.
-Technical Specifications
-Fabric CompositionPremium Cotton &amp; Technical Performance BlendFit ProfileModern Tailored Silhouette (True to Size)Care InstructionsMachine wash cold with like colors, tumble dry lowBrand OriginShockoeatelier (United States)CraftsmanshipReinforced Seams &amp; Colorfast Finish</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="n">
+        <v>371</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Agent-Optimized Item</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Crafted from premium 12.5oz Italian selvedge denim, the Ivy fit offers a relaxed yet refined silhouette that breaks in perfectly over time. These black-on-black jeans feature a unique slub character that adds deep texture and visual interest to every pair.
+Key Features &amp; Performance Specifications
+• Fabric: 12.5oz Italian Selvedge Denim from Candiani Mills
+• Fit: High rise with a relaxed seat and gentle taper
+• Construction: 100% Cotton with chain stitched hem
+• Hardware: Black coated copper rivets with leather backing
+• Value Add: Includes free lifetime repairs
+Weight: 12.5oz. Material: 100% Cotton. Color: Black/Black. Fit: Ivy (Relaxed/Tapered). Origin: Italy/USA.</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Ivy Black Selvedge - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="K5" s="9" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="M5" s="10" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Front view of black selvedge denim jeans showing the textured fabric, tonal stitching, and high-rise construction.</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Category:Denim, Fit:Ivy, Material:Cotton, Selvedge:Yes, Color:Black, Origin:USA, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>https://shockoeatelier.com/products/ivy-black-selvedge-100</t>
         </is>
@@ -913,53 +901,53 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Standard Black Selvedge | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
+          <t>Shockoe Atelier Standard Fit Black Selvedge Denim Jeans</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>269</v>
       </c>
-      <c r="F6" s="7" t="n">
-        <v>384</v>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Standard Catalog Item</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>The Standard Black Selvedge by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
-Key Features &amp; Highlights
-• Performance Fabric Blend: Engineered for superior breathability, natural stretch, and all-day comfort.
-• Tailored Precision Silhouette: Modern athletic profile that transitions seamlessly from office to active wear.
-• Reinforced Durability: Double-needle flatlock stitching on high-stress seams prevents warping and fraying.
-• Pre-Shrunk &amp; Easy Care: Maintains original fit, color depth, and soft hand-feel wash after wash.
-Technical Specifications
-Fabric CompositionPremium Cotton &amp; Technical Performance BlendFit ProfileModern Tailored Silhouette (True to Size)Care InstructionsMachine wash cold with like colors, tumble dry lowBrand OriginShockoeatelier (United States)CraftsmanshipReinforced Seams &amp; Colorfast Finish</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Agent-Optimized Item</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>The Standard Fit black selvedge denim combines a versatile silhouette with high-quality Italian construction designed to mold uniquely to your body. These jeans serve as a durable, timeless wardrobe staple that transitions effortlessly from the workshop to a night out.
+Key Features &amp; Performance Specifications
+• Fabric: 12.5oz Italian Selvedge Denim from Candiani Mills
+• Fit: Low-Mid rise with a trim, versatile silhouette
+• Construction: 100% Cotton with lined back pockets
+• Hardware: Black coated copper rivets with leather backing
+• Value Add: Includes free lifetime repairs
+Weight: 12.5oz. Material: 100% Cotton. Color: Black/Black. Fit: Standard. Origin: Italy/USA.</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>Standard Black Selvedge - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="K6" s="9" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Profile view of standard black selvedge denim jeans highlighting the tapered leg, clean lines, and premium copper hardware.</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Category:Denim, Fit:Standard, Material:Cotton, Selvedge:Yes, Color:Black, Origin:USA, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
         <is>
           <t>https://shockoeatelier.com/products/standard-black-selvedge-100</t>
         </is>
@@ -967,11 +955,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1018,892 +1006,842 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Handle</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Body (HTML)</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Product Category</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Option1 Name</t>
         </is>
       </c>
-      <c r="J1" s="11" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Option1 Value</t>
         </is>
       </c>
-      <c r="K1" s="11" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Variant SKU</t>
         </is>
       </c>
-      <c r="L1" s="11" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Variant Grams</t>
         </is>
       </c>
-      <c r="M1" s="11" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Variant Inventory Tracker</t>
         </is>
       </c>
-      <c r="N1" s="11" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Variant Inventory Qty</t>
         </is>
       </c>
-      <c r="O1" s="11" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>Variant Inventory Policy</t>
         </is>
       </c>
-      <c r="P1" s="11" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>Variant Fulfillment Service</t>
         </is>
       </c>
-      <c r="Q1" s="11" t="inlineStr">
+      <c r="Q1" s="8" t="inlineStr">
         <is>
           <t>Variant Price</t>
         </is>
       </c>
-      <c r="R1" s="11" t="inlineStr">
+      <c r="R1" s="8" t="inlineStr">
         <is>
           <t>Variant Compare At Price</t>
         </is>
       </c>
-      <c r="S1" s="11" t="inlineStr">
+      <c r="S1" s="8" t="inlineStr">
         <is>
           <t>Variant Requires Shipping</t>
         </is>
       </c>
-      <c r="T1" s="11" t="inlineStr">
+      <c r="T1" s="8" t="inlineStr">
         <is>
           <t>Variant Taxable</t>
         </is>
       </c>
-      <c r="U1" s="11" t="inlineStr">
+      <c r="U1" s="8" t="inlineStr">
         <is>
           <t>Variant Barcode</t>
         </is>
       </c>
-      <c r="V1" s="11" t="inlineStr">
+      <c r="V1" s="8" t="inlineStr">
         <is>
           <t>Image Src</t>
         </is>
       </c>
-      <c r="W1" s="11" t="inlineStr">
+      <c r="W1" s="8" t="inlineStr">
         <is>
           <t>Image Position</t>
         </is>
       </c>
-      <c r="X1" s="11" t="inlineStr">
+      <c r="X1" s="8" t="inlineStr">
         <is>
           <t>Image Alt Text</t>
         </is>
       </c>
-      <c r="Y1" s="11" t="inlineStr">
+      <c r="Y1" s="8" t="inlineStr">
         <is>
           <t>Gift Card</t>
         </is>
       </c>
-      <c r="Z1" s="11" t="inlineStr">
+      <c r="Z1" s="8" t="inlineStr">
         <is>
           <t>SEO Title</t>
         </is>
       </c>
-      <c r="AA1" s="11" t="inlineStr">
+      <c r="AA1" s="8" t="inlineStr">
         <is>
           <t>SEO Description</t>
         </is>
       </c>
-      <c r="AB1" s="11" t="inlineStr">
+      <c r="AB1" s="8" t="inlineStr">
         <is>
           <t>Google Shopping / Google Product Category</t>
         </is>
       </c>
-      <c r="AC1" s="11" t="inlineStr">
+      <c r="AC1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>room-spray</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>High Point Originals Room Spray | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The &lt;strong&gt;High Point Originals Room Spray&lt;/strong&gt; by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
-&lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
-&lt;ul style='padding-left:20px; line-height:1.6;'&gt;
-&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Performance Fabric Blend:&lt;/strong&gt; Engineered for superior breathability, natural stretch, and all-day comfort.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Tailored Precision Silhouette:&lt;/strong&gt; Modern athletic profile that transitions seamlessly from office to active wear.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Reinforced Durability:&lt;/strong&gt; Double-needle flatlock stitching on high-stress seams prevents warping and fraying.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Pre-Shrunk &amp; Easy Care:&lt;/strong&gt; Maintains original fit, color depth, and soft hand-feel wash after wash.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Technical Specifications&lt;/h3&gt;
-&lt;table style='width:100%; border-collapse:collapse; margin-top:12px; font-size:14px; text-align:left;'&gt;
-  &lt;tbody&gt;
-&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fabric Composition&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Premium Cotton &amp; Technical Performance Blend&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fit Profile&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Modern Tailored Silhouette (True to Size)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Care Instructions&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Machine wash cold with like colors, tumble dry low&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Brand Origin&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Shockoeatelier (United States)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Craftsmanship&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Reinforced Seams &amp; Colorfast Finish&lt;/td&gt;&lt;/tr&gt;
-  &lt;/tbody&gt;
-&lt;/table&gt;</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>High Point Originals Meadow Street Signature Room Spray</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Instantly transform your home environment with the sophisticated, crisp scent of High Point Barber Shop's signature Meadow Street fragrance. Designed for those who value refined living, this premium spray provides a lasting aromatic experience that elevates any room's atmosphere.&lt;/p&gt;&lt;h3&gt;Key Features &amp; Performance Specifications&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Fragrance Profile:&lt;/strong&gt; Meadow Street signature botanical blend&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Application:&lt;/strong&gt; Instant mist for home, office, or linens&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Concentration:&lt;/strong&gt; Long-lasting premium aromatic formulation&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design:&lt;/strong&gt; Minimalist apothecary-style glass bottle&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Origin:&lt;/strong&gt; Hand-crafted in the USA&lt;/li&gt;&lt;/ul&gt;&lt;div class="specs-summary"&gt;&lt;p&gt;Materials: Glass bottle, aromatic essential oils. Care: Spray away from face and delicate fabrics. Origin: USA.&lt;/p&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>Shockoeatelier</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="G2" s="12" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden &gt; Decor &gt; Home Fragrance &gt; Room Sprays</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden &gt; Decor &gt; Home Fragrance &gt; Room Sprays</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>Category:Home Fragrance, Scent:Meadow Street, Style:Apothecary, Material:Glass, Usage:Aromatherapy, Brand:High Point Originals, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>ROOM-SPRAY-FIXED</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P2" s="12" t="inlineStr">
+      <c r="P2" s="9" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="Q2" s="9" t="inlineStr">
         <is>
           <t>3400.00</t>
         </is>
       </c>
-      <c r="R2" s="12" t="inlineStr"/>
-      <c r="S2" s="12" t="inlineStr">
+      <c r="R2" s="9" t="inlineStr"/>
+      <c r="S2" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T2" s="12" t="inlineStr">
+      <c r="T2" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U2" s="12" t="inlineStr"/>
-      <c r="V2" s="12" t="inlineStr">
+      <c r="U2" s="9" t="inlineStr"/>
+      <c r="V2" s="9" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0216/3732/products/rs_bottle.jpg?v=1655306746</t>
         </is>
       </c>
-      <c r="W2" s="12" t="inlineStr">
+      <c r="W2" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X2" s="12" t="inlineStr">
-        <is>
-          <t>High Point Originals Room Spray - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="Y2" s="12" t="inlineStr">
+      <c r="X2" s="9" t="inlineStr">
+        <is>
+          <t>A clear glass bottle of High Point Originals Meadow Street room spray featuring a minimalist white label, set against a neutral studio background.</t>
+        </is>
+      </c>
+      <c r="Y2" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z2" s="12" t="inlineStr">
-        <is>
-          <t>High Point Originals Room Spray | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="AA2" s="12" t="inlineStr">
-        <is>
-          <t>The  High Point Originals Room Spray  by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully en</t>
-        </is>
-      </c>
-      <c r="AB2" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="AC2" s="12" t="inlineStr">
+      <c r="Z2" s="9" t="inlineStr">
+        <is>
+          <t>High Point Originals Meadow Street Signature Room Spray</t>
+        </is>
+      </c>
+      <c r="AA2" s="9" t="inlineStr">
+        <is>
+          <t>Instantly transform your home environment with the sophisticated, crisp scent of High Point Barber Shop's signature Meadow Street fragrance. Designed for t</t>
+        </is>
+      </c>
+      <c r="AB2" s="9" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden &gt; Decor &gt; Home Fragrance &gt; Room Sprays</t>
+        </is>
+      </c>
+      <c r="AC2" s="9" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>50-gift-card</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Gift Card | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The &lt;strong&gt;Gift Card&lt;/strong&gt; by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
-&lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
-&lt;ul style='padding-left:20px; line-height:1.6;'&gt;
-&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Performance Fabric Blend:&lt;/strong&gt; Engineered for superior breathability, natural stretch, and all-day comfort.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Tailored Precision Silhouette:&lt;/strong&gt; Modern athletic profile that transitions seamlessly from office to active wear.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Reinforced Durability:&lt;/strong&gt; Double-needle flatlock stitching on high-stress seams prevents warping and fraying.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Pre-Shrunk &amp; Easy Care:&lt;/strong&gt; Maintains original fit, color depth, and soft hand-feel wash after wash.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Technical Specifications&lt;/h3&gt;
-&lt;table style='width:100%; border-collapse:collapse; margin-top:12px; font-size:14px; text-align:left;'&gt;
-  &lt;tbody&gt;
-&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fabric Composition&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Premium Cotton &amp; Technical Performance Blend&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fit Profile&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Modern Tailored Silhouette (True to Size)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Care Instructions&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Machine wash cold with like colors, tumble dry low&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Brand Origin&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Shockoeatelier (United States)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Craftsmanship&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Reinforced Seams &amp; Colorfast Finish&lt;/td&gt;&lt;/tr&gt;
-  &lt;/tbody&gt;
-&lt;/table&gt;</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Shockoe Atelier Digital &amp; Physical Gift Card</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Give the gift of choice with a versatile Shockoe Atelier gift card, perfect for the denim enthusiast or modern minimalist in your life. Our gift cards are delivered seamlessly via email for immediate use or available as a premium physical card for a more personal touch.&lt;/p&gt;&lt;h3&gt;Key Features &amp; Performance Specifications&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Flexibility:&lt;/strong&gt; Redeemable storewide for all apparel and accessories&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Delivery Options:&lt;/strong&gt; Immediate email delivery or physical mail&lt;/li&gt;&lt;li&gt;&lt;strong&gt;No Expiration:&lt;/strong&gt; Credit never expires for user convenience&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Personalization:&lt;/strong&gt; Physical cards available upon request&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Customer Support:&lt;/strong&gt; Dedicated assistance via info@shockoeatelier.com&lt;/li&gt;&lt;/ul&gt;&lt;div class="specs-summary"&gt;&lt;p&gt;Format: Digital/Physical. Compatibility: All products online and in-store. Origin: Shockoe Atelier.&lt;/p&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Shockoeatelier</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Gift Cards</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Gift Cards</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Category:Gift Card, Occasion:Gift, Brand:Shockoe Atelier, Format:Digital, Format:Physical, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K3" s="12" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>50-GIFT-CARD-FIXED</t>
         </is>
       </c>
-      <c r="L3" s="12" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M3" s="12" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N3" s="12" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O3" s="12" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P3" s="12" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>6572.14</t>
         </is>
       </c>
-      <c r="R3" s="12" t="inlineStr"/>
-      <c r="S3" s="12" t="inlineStr">
+      <c r="R3" s="9" t="inlineStr"/>
+      <c r="S3" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T3" s="12" t="inlineStr">
+      <c r="T3" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U3" s="12" t="inlineStr"/>
-      <c r="V3" s="12" t="inlineStr">
+      <c r="U3" s="9" t="inlineStr"/>
+      <c r="V3" s="9" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0216/3732/products/201201-giftcard-1.1_18cc2655-be22-47c2-a4b6-cf6fca6f2a7f.jpg?v=1608079723</t>
         </is>
       </c>
-      <c r="W3" s="12" t="inlineStr">
+      <c r="W3" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X3" s="12" t="inlineStr">
-        <is>
-          <t>Gift Card - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="Y3" s="12" t="inlineStr">
+      <c r="X3" s="9" t="inlineStr">
+        <is>
+          <t>A physical Shockoe Atelier branded gift card displayed on a clean wooden surface, symbolizing premium quality and choice.</t>
+        </is>
+      </c>
+      <c r="Y3" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z3" s="12" t="inlineStr">
-        <is>
-          <t>Gift Card | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="AA3" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The  Gift Card  by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate </t>
-        </is>
-      </c>
-      <c r="AB3" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="AC3" s="12" t="inlineStr">
+      <c r="Z3" s="9" t="inlineStr">
+        <is>
+          <t>Shockoe Atelier Digital &amp; Physical Gift Card</t>
+        </is>
+      </c>
+      <c r="AA3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Give the gift of choice with a versatile Shockoe Atelier gift card, perfect for the denim enthusiast or modern minimalist in your life. Our gift cards are </t>
+        </is>
+      </c>
+      <c r="AB3" s="9" t="inlineStr">
+        <is>
+          <t>Gift Cards</t>
+        </is>
+      </c>
+      <c r="AC3" s="9" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>billy-made-for-friends-brass-cuff</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Billy Made For Friends Thin Brass Bar Cuff | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The &lt;strong&gt;Billy Made For Friends Thin Brass Bar Cuff&lt;/strong&gt; by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
-&lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
-&lt;ul style='padding-left:20px; line-height:1.6;'&gt;
-&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Performance Fabric Blend:&lt;/strong&gt; Engineered for superior breathability, natural stretch, and all-day comfort.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Tailored Precision Silhouette:&lt;/strong&gt; Modern athletic profile that transitions seamlessly from office to active wear.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Reinforced Durability:&lt;/strong&gt; Double-needle flatlock stitching on high-stress seams prevents warping and fraying.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Pre-Shrunk &amp; Easy Care:&lt;/strong&gt; Maintains original fit, color depth, and soft hand-feel wash after wash.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Technical Specifications&lt;/h3&gt;
-&lt;table style='width:100%; border-collapse:collapse; margin-top:12px; font-size:14px; text-align:left;'&gt;
-  &lt;tbody&gt;
-&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fabric Composition&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Premium Cotton &amp; Technical Performance Blend&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fit Profile&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Modern Tailored Silhouette (True to Size)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Care Instructions&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Machine wash cold with like colors, tumble dry low&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Brand Origin&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Shockoeatelier (United States)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Craftsmanship&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Reinforced Seams &amp; Colorfast Finish&lt;/td&gt;&lt;/tr&gt;
-  &lt;/tbody&gt;
-&lt;/table&gt;</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Billy Made For Friends Textured Thin Brass Cuff Bracelet</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Add a touch of rugged, artisanal detail to your wrist with this thin brass cuff, hand-finished by master craftsman Billy Moore in Asheville, NC. Its subtle texture offers a unique, worn-in aesthetic that complements any casual or tailored wardrobe.&lt;/p&gt;&lt;h3&gt;Key Features &amp; Performance Specifications&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Material:&lt;/strong&gt; 100% solid, high-grade &lt;strong&gt;Brass&lt;/strong&gt;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Design:&lt;/strong&gt; Slim profile with unique &lt;strong&gt;textured finish&lt;/strong&gt;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Craftsmanship:&lt;/strong&gt; Handmade in the USA by Billy Moore&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Style:&lt;/strong&gt; Minimalist, gender-neutral jewelry piece&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Durability:&lt;/strong&gt; Develops a rich natural patina over time&lt;/li&gt;&lt;/ul&gt;&lt;div class="specs-summary"&gt;&lt;p&gt;Material: Solid Brass. Construction: Handmade. Finish: Textured. Origin: USA. Size: One size adjustable.&lt;/p&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Shockoeatelier</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Jewelry &gt; Bracelets</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Jewelry &gt; Bracelets</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Category:Jewelry, Material:Brass, Style:Minimalist, Origin:USA, Product:Cuff Bracelet, Gender:Unisex, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>BILLY-MADE-FOR-FRIEN-FIXED</t>
         </is>
       </c>
-      <c r="L4" s="12" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M4" s="12" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N4" s="12" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O4" s="12" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P4" s="12" t="inlineStr">
+      <c r="P4" s="9" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q4" s="12" t="inlineStr">
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>8700.00</t>
         </is>
       </c>
-      <c r="R4" s="12" t="inlineStr"/>
-      <c r="S4" s="12" t="inlineStr">
+      <c r="R4" s="9" t="inlineStr"/>
+      <c r="S4" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T4" s="12" t="inlineStr">
+      <c r="T4" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U4" s="12" t="inlineStr"/>
-      <c r="V4" s="12" t="inlineStr">
+      <c r="U4" s="9" t="inlineStr"/>
+      <c r="V4" s="9" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0216/3732/files/9.jpg?v=1753213737</t>
         </is>
       </c>
-      <c r="W4" s="12" t="inlineStr">
+      <c r="W4" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X4" s="12" t="inlineStr">
-        <is>
-          <t>Billy Made For Friends Thin Brass Bar Cuff - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="Y4" s="12" t="inlineStr">
+      <c r="X4" s="9" t="inlineStr">
+        <is>
+          <t>Close-up macro shot of a thin, textured brass cuff bracelet showing the fine metallic details and artisanal finish.</t>
+        </is>
+      </c>
+      <c r="Y4" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z4" s="12" t="inlineStr">
-        <is>
-          <t>Billy Made For Friends Thin Brass Bar Cuff | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="AA4" s="12" t="inlineStr">
-        <is>
-          <t>The  Billy Made For Friends Thin Brass Bar Cuff  by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thou</t>
-        </is>
-      </c>
-      <c r="AB4" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="AC4" s="12" t="inlineStr">
+      <c r="Z4" s="9" t="inlineStr">
+        <is>
+          <t>Billy Made For Friends Textured Thin Brass Cuff Bracelet</t>
+        </is>
+      </c>
+      <c r="AA4" s="9" t="inlineStr">
+        <is>
+          <t>Add a touch of rugged, artisanal detail to your wrist with this thin brass cuff, hand-finished by master craftsman Billy Moore in Asheville, NC. Its subtle</t>
+        </is>
+      </c>
+      <c r="AB4" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Jewelry &gt; Bracelets</t>
+        </is>
+      </c>
+      <c r="AC4" s="9" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>ivy-black-selvedge-100</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Ivy Black Selvedge | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The &lt;strong&gt;Ivy Black Selvedge&lt;/strong&gt; by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
-&lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
-&lt;ul style='padding-left:20px; line-height:1.6;'&gt;
-&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Performance Fabric Blend:&lt;/strong&gt; Engineered for superior breathability, natural stretch, and all-day comfort.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Tailored Precision Silhouette:&lt;/strong&gt; Modern athletic profile that transitions seamlessly from office to active wear.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Reinforced Durability:&lt;/strong&gt; Double-needle flatlock stitching on high-stress seams prevents warping and fraying.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Pre-Shrunk &amp; Easy Care:&lt;/strong&gt; Maintains original fit, color depth, and soft hand-feel wash after wash.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Technical Specifications&lt;/h3&gt;
-&lt;table style='width:100%; border-collapse:collapse; margin-top:12px; font-size:14px; text-align:left;'&gt;
-  &lt;tbody&gt;
-&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fabric Composition&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Premium Cotton &amp; Technical Performance Blend&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fit Profile&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Modern Tailored Silhouette (True to Size)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Care Instructions&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Machine wash cold with like colors, tumble dry low&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Brand Origin&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Shockoeatelier (United States)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Craftsmanship&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Reinforced Seams &amp; Colorfast Finish&lt;/td&gt;&lt;/tr&gt;
-  &lt;/tbody&gt;
-&lt;/table&gt;</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Shockoe Atelier Ivy Fit Black Selvedge Denim Jeans</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Crafted from premium 12.5oz Italian selvedge denim, the Ivy fit offers a relaxed yet refined silhouette that breaks in perfectly over time. These black-on-black jeans feature a unique slub character that adds deep texture and visual interest to every pair.&lt;/p&gt;&lt;h3&gt;Key Features &amp; Performance Specifications&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Fabric:&lt;/strong&gt; 12.5oz &lt;strong&gt;Italian Selvedge Denim&lt;/strong&gt; from Candiani Mills&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Fit:&lt;/strong&gt; &lt;strong&gt;High rise&lt;/strong&gt; with a relaxed seat and gentle taper&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Construction:&lt;/strong&gt; 100% Cotton with &lt;strong&gt;chain stitched hem&lt;/strong&gt;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Hardware:&lt;/strong&gt; Black coated copper rivets with &lt;strong&gt;leather backing&lt;/strong&gt;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Value Add:&lt;/strong&gt; Includes &lt;strong&gt;free lifetime repairs&lt;/strong&gt;&lt;/li&gt;&lt;/ul&gt;&lt;div class="specs-summary"&gt;&lt;p&gt;Weight: 12.5oz. Material: 100% Cotton. Color: Black/Black. Fit: Ivy (Relaxed/Tapered). Origin: Italy/USA.&lt;/p&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Shockoeatelier</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Category:Denim, Fit:Ivy, Material:Cotton, Selvedge:Yes, Color:Black, Origin:USA, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>IVY-BLACK-SELVEDGE-1-FIXED</t>
         </is>
       </c>
-      <c r="L5" s="12" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M5" s="12" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N5" s="12" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O5" s="12" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P5" s="12" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="inlineStr">
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>36700.00</t>
         </is>
       </c>
-      <c r="R5" s="12" t="inlineStr"/>
-      <c r="S5" s="12" t="inlineStr">
+      <c r="R5" s="9" t="inlineStr"/>
+      <c r="S5" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T5" s="12" t="inlineStr">
+      <c r="T5" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U5" s="12" t="inlineStr"/>
-      <c r="V5" s="12" t="inlineStr">
+      <c r="U5" s="9" t="inlineStr"/>
+      <c r="V5" s="9" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0216/3732/files/Shokoe1-22-2516957.jpg?v=1770388499</t>
         </is>
       </c>
-      <c r="W5" s="12" t="inlineStr">
+      <c r="W5" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X5" s="12" t="inlineStr">
-        <is>
-          <t>Ivy Black Selvedge - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="Y5" s="12" t="inlineStr">
+      <c r="X5" s="9" t="inlineStr">
+        <is>
+          <t>Front view of black selvedge denim jeans showing the textured fabric, tonal stitching, and high-rise construction.</t>
+        </is>
+      </c>
+      <c r="Y5" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z5" s="12" t="inlineStr">
-        <is>
-          <t>Ivy Black Selvedge | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="AA5" s="12" t="inlineStr">
-        <is>
-          <t>The  Ivy Black Selvedge  by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to e</t>
-        </is>
-      </c>
-      <c r="AB5" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="AC5" s="12" t="inlineStr">
+      <c r="Z5" s="9" t="inlineStr">
+        <is>
+          <t>Shockoe Atelier Ivy Fit Black Selvedge Denim Jeans</t>
+        </is>
+      </c>
+      <c r="AA5" s="9" t="inlineStr">
+        <is>
+          <t>Crafted from premium 12.5oz Italian selvedge denim, the Ivy fit offers a relaxed yet refined silhouette that breaks in perfectly over time. These black-on-</t>
+        </is>
+      </c>
+      <c r="AB5" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="AC5" s="9" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>standard-black-selvedge-100</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Standard Black Selvedge | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The &lt;strong&gt;Standard Black Selvedge&lt;/strong&gt; by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
-&lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
-&lt;ul style='padding-left:20px; line-height:1.6;'&gt;
-&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Performance Fabric Blend:&lt;/strong&gt; Engineered for superior breathability, natural stretch, and all-day comfort.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Tailored Precision Silhouette:&lt;/strong&gt; Modern athletic profile that transitions seamlessly from office to active wear.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Reinforced Durability:&lt;/strong&gt; Double-needle flatlock stitching on high-stress seams prevents warping and fraying.&lt;/li&gt;&lt;li style='margin-bottom:6px;'&gt;&lt;strong&gt;Pre-Shrunk &amp; Easy Care:&lt;/strong&gt; Maintains original fit, color depth, and soft hand-feel wash after wash.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Technical Specifications&lt;/h3&gt;
-&lt;table style='width:100%; border-collapse:collapse; margin-top:12px; font-size:14px; text-align:left;'&gt;
-  &lt;tbody&gt;
-&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fabric Composition&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Premium Cotton &amp; Technical Performance Blend&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Fit Profile&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Modern Tailored Silhouette (True to Size)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Care Instructions&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Machine wash cold with like colors, tumble dry low&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Brand Origin&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Shockoeatelier (United States)&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0; font-weight:600; background:#f8fafc; width:35%;'&gt;Craftsmanship&lt;/td&gt;&lt;td style='padding:6px 10px; border:1px solid #e2e8f0;'&gt;Reinforced Seams &amp; Colorfast Finish&lt;/td&gt;&lt;/tr&gt;
-  &lt;/tbody&gt;
-&lt;/table&gt;</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Shockoe Atelier Standard Fit Black Selvedge Denim Jeans</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;The Standard Fit black selvedge denim combines a versatile silhouette with high-quality Italian construction designed to mold uniquely to your body. These jeans serve as a durable, timeless wardrobe staple that transitions effortlessly from the workshop to a night out.&lt;/p&gt;&lt;h3&gt;Key Features &amp; Performance Specifications&lt;/h3&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Fabric:&lt;/strong&gt; 12.5oz &lt;strong&gt;Italian Selvedge Denim&lt;/strong&gt; from Candiani Mills&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Fit:&lt;/strong&gt; &lt;strong&gt;Low-Mid rise&lt;/strong&gt; with a trim, versatile silhouette&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Construction:&lt;/strong&gt; 100% Cotton with &lt;strong&gt;lined back pockets&lt;/strong&gt;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Hardware:&lt;/strong&gt; Black coated copper rivets with &lt;strong&gt;leather backing&lt;/strong&gt;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Value Add:&lt;/strong&gt; Includes &lt;strong&gt;free lifetime repairs&lt;/strong&gt;&lt;/li&gt;&lt;/ul&gt;&lt;div class="specs-summary"&gt;&lt;p&gt;Weight: 12.5oz. Material: 100% Cotton. Color: Black/Black. Fit: Standard. Origin: Italy/USA.&lt;/p&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Shockoeatelier</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>Apparel, Everyday Wear, Performance Fit, Premium Essentials, Made in USA, Tailored Collection</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Category:Denim, Fit:Standard, Material:Cotton, Selvedge:Yes, Color:Black, Origin:USA, Agentic:Ready</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>STANDARD-BLACK-SELVE-FIXED</t>
         </is>
       </c>
-      <c r="L6" s="12" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M6" s="12" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N6" s="12" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O6" s="12" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P6" s="12" t="inlineStr">
+      <c r="P6" s="9" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>36700.00</t>
         </is>
       </c>
-      <c r="R6" s="12" t="inlineStr"/>
-      <c r="S6" s="12" t="inlineStr">
+      <c r="R6" s="9" t="inlineStr"/>
+      <c r="S6" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T6" s="12" t="inlineStr">
+      <c r="T6" s="9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U6" s="12" t="inlineStr"/>
-      <c r="V6" s="12" t="inlineStr">
+      <c r="U6" s="9" t="inlineStr"/>
+      <c r="V6" s="9" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0216/3732/files/Shokoe1-22-2517024.jpg?v=1770388372</t>
         </is>
       </c>
-      <c r="W6" s="12" t="inlineStr">
+      <c r="W6" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X6" s="12" t="inlineStr">
-        <is>
-          <t>Standard Black Selvedge - Shockoeatelier Official Product View</t>
-        </is>
-      </c>
-      <c r="Y6" s="12" t="inlineStr">
+      <c r="X6" s="9" t="inlineStr">
+        <is>
+          <t>Profile view of standard black selvedge denim jeans highlighting the tapered leg, clean lines, and premium copper hardware.</t>
+        </is>
+      </c>
+      <c r="Y6" s="9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z6" s="12" t="inlineStr">
-        <is>
-          <t>Standard Black Selvedge | Everyday Performance &amp; Fit</t>
-        </is>
-      </c>
-      <c r="AA6" s="12" t="inlineStr">
-        <is>
-          <t>The  Standard Black Selvedge  by Shockoeatelier represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered</t>
-        </is>
-      </c>
-      <c r="AB6" s="12" t="inlineStr">
-        <is>
-          <t>Apparel &amp; Accessories &gt; Clothing</t>
-        </is>
-      </c>
-      <c r="AC6" s="12" t="inlineStr">
+      <c r="Z6" s="9" t="inlineStr">
+        <is>
+          <t>Shockoe Atelier Standard Fit Black Selvedge Denim Jeans</t>
+        </is>
+      </c>
+      <c r="AA6" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Standard Fit black selvedge denim combines a versatile silhouette with high-quality Italian construction designed to mold uniquely to your body. These </t>
+        </is>
+      </c>
+      <c r="AB6" s="9" t="inlineStr">
+        <is>
+          <t>Apparel &amp; Accessories &gt; Clothing &gt; Pants</t>
+        </is>
+      </c>
+      <c r="AC6" s="9" t="inlineStr">
         <is>
           <t>draft</t>
         </is>

</xml_diff>